<commit_message>
Updated All Table Models
</commit_message>
<xml_diff>
--- a/Zenskar_MAMS/Helpers/Queries.xlsx
+++ b/Zenskar_MAMS/Helpers/Queries.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180" activeTab="2"/>
+    <workbookView windowWidth="28800" windowHeight="11460" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="89">
+  <si>
+    <t>Slno</t>
+  </si>
   <si>
     <t>FileName</t>
   </si>
@@ -65,6 +68,42 @@
 LoginUser1</t>
   </si>
   <si>
+    <t>Page</t>
+  </si>
+  <si>
+    <t>No. Queries</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Works</t>
+  </si>
+  <si>
+    <t>Commited</t>
+  </si>
+  <si>
+    <t>AdminHome</t>
+  </si>
+  <si>
+    <t>Attendance</t>
+  </si>
+  <si>
+    <t>FilterWindow</t>
+  </si>
+  <si>
+    <t>InstructorHome</t>
+  </si>
+  <si>
+    <t>MasterHome</t>
+  </si>
+  <si>
+    <t>Register</t>
+  </si>
+  <si>
+    <t>RejectReasonWindow</t>
+  </si>
+  <si>
     <t>RequestDetailsWindow</t>
   </si>
   <si>
@@ -81,30 +120,6 @@
   </si>
   <si>
     <t>UserManagement</t>
-  </si>
-  <si>
-    <t>AdminHome</t>
-  </si>
-  <si>
-    <t>Attendance</t>
-  </si>
-  <si>
-    <t>FilterWindow</t>
-  </si>
-  <si>
-    <t>InstructorHome</t>
-  </si>
-  <si>
-    <t>MasterHome</t>
-  </si>
-  <si>
-    <t>Register</t>
-  </si>
-  <si>
-    <t>RejectReasonWindow</t>
-  </si>
-  <si>
-    <t>Slno</t>
   </si>
   <si>
     <t>MongoFilter</t>
@@ -909,8 +924,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
@@ -1451,38 +1466,41 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="5"/>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="2" outlineLevelCol="6"/>
   <cols>
-    <col min="2" max="2" width="110.571428571429" customWidth="1"/>
-    <col min="3" max="3" width="11.4285714285714" customWidth="1"/>
-    <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="13.8571428571429" customWidth="1"/>
+    <col min="3" max="3" width="110.571428571429" customWidth="1"/>
+    <col min="4" max="4" width="11.4285714285714" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="6" max="6" width="13.8571428571429" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" ht="30" spans="1:6">
-      <c r="A2" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="2" ht="30" spans="1:7">
+      <c r="A2">
+        <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
@@ -1493,11 +1511,19 @@
       <c r="D2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" t="s">
-        <v>9</v>
+      <c r="F2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1509,83 +1535,165 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:A14"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="1" max="1" width="5.42857142857143" style="1" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="12.4285714285714" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5714285714286" style="1" customWidth="1"/>
+    <col min="5" max="5" width="9.14285714285714" style="1"/>
+    <col min="6" max="6" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="1">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="1">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:1">
-      <c r="A2" t="s">
+      <c r="B12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="1">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:1">
-      <c r="A3" t="s">
+      <c r="B13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="1">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" spans="1:1">
-      <c r="A4" t="s">
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" s="1">
         <v>14</v>
       </c>
-    </row>
-    <row r="5" spans="1:1">
-      <c r="A5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1">
-      <c r="A6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1">
-      <c r="A7" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1">
-      <c r="A8" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1">
-      <c r="A9" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1">
-      <c r="A10" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1">
-      <c r="A11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1">
-      <c r="A12" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1">
-      <c r="A13" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1">
-      <c r="A14" t="s">
-        <v>23</v>
+      <c r="B15" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
+  <sortState ref="B3:B15">
+    <sortCondition ref="B3"/>
+  </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
@@ -1607,19 +1715,19 @@
   <sheetData>
     <row r="1" customFormat="1" spans="1:5">
       <c r="A1" t="s">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -1627,19 +1735,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C2" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E2" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1647,19 +1755,19 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C3" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D3" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F3" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1667,19 +1775,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="E4" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F4" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1687,19 +1795,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="E5" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F5" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1707,19 +1815,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="E6" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F6" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1727,19 +1835,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="D7" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="E7" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="F7" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1747,19 +1855,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C8" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="D8" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="E8" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="F8" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1767,19 +1875,19 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C9" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="D9" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="E9" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F9" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1787,19 +1895,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C10" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="D10" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="E10" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F10" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1807,19 +1915,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C11" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="D11" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="E11" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="F11" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1827,19 +1935,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C12" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="D12" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="E12" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="F12" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1847,19 +1955,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C13" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D13" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E13" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F13" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -1867,19 +1975,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C14" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D14" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E14" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F14" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -1887,19 +1995,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C15" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="D15" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E15" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F15" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -1907,19 +2015,19 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C16" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="D16" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E16" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F16" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -1927,19 +2035,19 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C17" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="D17" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E17" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F17" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -1947,19 +2055,19 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C18" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="D18" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="E18" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="F18" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -1967,19 +2075,19 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C19" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="D19" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E19" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F19" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -1987,19 +2095,19 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C20" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="D20" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="E20" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="F20" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -2007,19 +2115,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C21" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="D21" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="E21" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="F21" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -2027,19 +2135,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C22" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="D22" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="E22" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="F22" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -2047,19 +2155,19 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C23" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D23" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E23" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F23" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -2067,19 +2175,19 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C24" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="D24" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E24" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F24" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -2087,19 +2195,19 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C25" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="D25" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E25" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F25" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -2107,19 +2215,19 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C26" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="D26" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="E26" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="F26" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -2127,19 +2235,19 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C27" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="D27" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="E27" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="F27" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -2147,19 +2255,19 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C28" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D28" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="E28" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="F28" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -2167,19 +2275,19 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C29" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="D29" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="E29" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="F29" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -2187,19 +2295,19 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C30" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="D30" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E30" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="F30" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -2207,19 +2315,19 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C31" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="D31" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E31" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F31" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -2227,19 +2335,19 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C32" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="D32" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="E32" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="F32" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -2247,19 +2355,19 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C33" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="D33" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="E33" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="F33" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -2267,19 +2375,19 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C34" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="D34" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E34" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F34" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -2287,19 +2395,19 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C35" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="D35" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E35" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F35" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -2307,19 +2415,19 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C36" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D36" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E36" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="F36" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -2327,19 +2435,19 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C37" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D37" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E37" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F37" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -2347,19 +2455,19 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C38" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="D38" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E38" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F38" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -2367,19 +2475,19 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C39" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="D39" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="E39" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="F39" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -2387,19 +2495,19 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="C40" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="D40" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="E40" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="F40" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -2407,19 +2515,19 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C41" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="D41" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E41" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="F41" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -2427,19 +2535,19 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C42" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D42" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E42" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F42" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Users Page rewrite InProgress
</commit_message>
<xml_diff>
--- a/Zenskar_MAMS/Helpers/Queries.xlsx
+++ b/Zenskar_MAMS/Helpers/Queries.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21000" windowHeight="8400" activeTab="1"/>
+    <workbookView windowWidth="21000" windowHeight="7680" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="111">
   <si>
     <t>Slno</t>
   </si>
@@ -192,6 +192,9 @@
   </si>
   <si>
     <t>UserManagement</t>
+  </si>
+  <si>
+    <t>1 select has if based conditions</t>
   </si>
   <si>
     <t>Total</t>
@@ -2133,16 +2136,16 @@
         <v>3</v>
       </c>
       <c r="H8" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I8" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J8" s="4"/>
       <c r="K8" s="4"/>
       <c r="L8" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Yet to be completed</v>
+        <v>Page completed</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -2201,7 +2204,7 @@
         <v>0</v>
       </c>
       <c r="G10" s="5">
-        <f>SUM(C10:F10)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H10" s="3">
@@ -2232,8 +2235,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
+      <c r="H11" s="3">
+        <v>0</v>
+      </c>
+      <c r="I11" s="3">
+        <v>0</v>
+      </c>
       <c r="J11" s="4"/>
       <c r="K11" s="13" t="s">
         <v>45</v>
@@ -2258,8 +2265,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
+      <c r="H12" s="3">
+        <v>0</v>
+      </c>
+      <c r="I12" s="3">
+        <v>0</v>
+      </c>
       <c r="J12" s="4"/>
       <c r="K12" s="4"/>
       <c r="L12" s="4" t="str">
@@ -2282,8 +2293,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
+      <c r="H13" s="3">
+        <v>0</v>
+      </c>
+      <c r="I13" s="3">
+        <v>0</v>
+      </c>
       <c r="J13" s="4"/>
       <c r="K13" s="4"/>
       <c r="L13" s="4" t="str">
@@ -2306,8 +2321,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
+      <c r="H14" s="3">
+        <v>0</v>
+      </c>
+      <c r="I14" s="3">
+        <v>0</v>
+      </c>
       <c r="J14" s="4"/>
       <c r="K14" s="13" t="s">
         <v>49</v>
@@ -2324,18 +2343,30 @@
       <c r="B15" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="C15" s="6"/>
+      <c r="C15" s="6">
+        <v>3</v>
+      </c>
       <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
+      <c r="E15" s="6">
+        <v>2</v>
+      </c>
+      <c r="F15" s="6">
+        <v>1</v>
+      </c>
       <c r="G15" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H15" s="8"/>
-      <c r="I15" s="8"/>
+        <v>6</v>
+      </c>
+      <c r="H15" s="8">
+        <v>4</v>
+      </c>
+      <c r="I15" s="8">
+        <v>4</v>
+      </c>
       <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
+      <c r="K15" s="4" t="s">
+        <v>51</v>
+      </c>
       <c r="L15" s="4" t="str">
         <f t="shared" si="1"/>
         <v>Yet to be completed</v>
@@ -2344,11 +2375,11 @@
     <row r="16" ht="15.15" spans="1:12">
       <c r="A16" s="9"/>
       <c r="B16" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C16" s="11">
         <f>SUM(C2:C15)</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D16" s="11">
         <f t="shared" ref="D16:I16" si="2">SUM(D2:D15)</f>
@@ -2356,23 +2387,23 @@
       </c>
       <c r="E16" s="11">
         <f t="shared" si="2"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F16" s="11">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" s="11">
         <f t="shared" si="2"/>
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="H16" s="11">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="I16" s="14">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="J16" s="15"/>
       <c r="K16" s="4"/>
@@ -2415,7 +2446,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -2423,19 +2454,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -2443,19 +2474,19 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -2463,19 +2494,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -2483,19 +2514,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C5" t="s">
+        <v>63</v>
+      </c>
+      <c r="D5" t="s">
         <v>62</v>
       </c>
-      <c r="D5" t="s">
-        <v>61</v>
-      </c>
       <c r="E5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -2503,19 +2534,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -2523,19 +2554,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -2543,19 +2574,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C8" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -2563,19 +2594,19 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C9" t="s">
         <v>19</v>
       </c>
       <c r="D9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -2583,19 +2614,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C10" t="s">
+        <v>72</v>
+      </c>
+      <c r="D10" t="s">
         <v>71</v>
       </c>
-      <c r="D10" t="s">
-        <v>70</v>
-      </c>
       <c r="E10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2603,19 +2634,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C11" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2623,19 +2654,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -2643,19 +2674,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -2663,19 +2694,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C14" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -2683,19 +2714,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C15" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F15" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -2703,19 +2734,19 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C16" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D16" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E16" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F16" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -2723,19 +2754,19 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C17" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D17" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E17" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F17" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -2743,19 +2774,19 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D18" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E18" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F18" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -2763,19 +2794,19 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C19" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D19" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E19" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F19" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -2783,19 +2814,19 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C20" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D20" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E20" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -2803,19 +2834,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C21" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D21" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E21" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F21" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -2823,19 +2854,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C22" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D22" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E22" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F22" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -2843,19 +2874,19 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C23" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D23" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E23" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F23" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -2863,19 +2894,19 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C24" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D24" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E24" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F24" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -2883,19 +2914,19 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C25" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D25" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E25" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F25" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -2903,19 +2934,19 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C26" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D26" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E26" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F26" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -2923,19 +2954,19 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C27" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D27" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E27" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F27" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -2943,19 +2974,19 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C28" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D28" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E28" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F28" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -2963,19 +2994,19 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C29" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D29" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E29" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F29" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -2983,19 +3014,19 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C30" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D30" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E30" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F30" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -3003,19 +3034,19 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C31" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D31" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E31" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F31" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -3023,19 +3054,19 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C32" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D32" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E32" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F32" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -3043,19 +3074,19 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C33" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D33" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E33" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F33" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -3063,19 +3094,19 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C34" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D34" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E34" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F34" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -3083,19 +3114,19 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C35" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D35" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E35" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F35" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -3103,19 +3134,19 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
+        <v>96</v>
+      </c>
+      <c r="C36" t="s">
+        <v>102</v>
+      </c>
+      <c r="D36" t="s">
         <v>95</v>
       </c>
-      <c r="C36" t="s">
-        <v>101</v>
-      </c>
-      <c r="D36" t="s">
-        <v>94</v>
-      </c>
       <c r="E36" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F36" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -3123,19 +3154,19 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C37" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D37" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E37" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F37" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -3143,19 +3174,19 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C38" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D38" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E38" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F38" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -3163,19 +3194,19 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C39" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D39" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E39" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F39" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -3183,19 +3214,19 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C40" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D40" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E40" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F40" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -3203,19 +3234,19 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C41" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D41" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E41" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F41" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -3223,19 +3254,19 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C42" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D42" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E42" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F42" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Completed UserMgmt Mongo Changes
</commit_message>
<xml_diff>
--- a/Zenskar_MAMS/Helpers/Queries.xlsx
+++ b/Zenskar_MAMS/Helpers/Queries.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21000" windowHeight="7680" activeTab="1"/>
+    <workbookView windowWidth="23040" windowHeight="8280" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2358,10 +2358,10 @@
         <v>6</v>
       </c>
       <c r="H15" s="8">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I15" s="8">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J15" s="4"/>
       <c r="K15" s="4" t="s">
@@ -2369,7 +2369,7 @@
       </c>
       <c r="L15" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Yet to be completed</v>
+        <v>Page completed</v>
       </c>
     </row>
     <row r="16" ht="15.15" spans="1:12">
@@ -2399,11 +2399,11 @@
       </c>
       <c r="H16" s="11">
         <f t="shared" si="2"/>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="I16" s="14">
         <f t="shared" si="2"/>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="J16" s="15"/>
       <c r="K16" s="4"/>

</xml_diff>

<commit_message>
Student Details 2 select completed
</commit_message>
<xml_diff>
--- a/Zenskar_MAMS/Helpers/Queries.xlsx
+++ b/Zenskar_MAMS/Helpers/Queries.xlsx
@@ -11,6 +11,9 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sheet2!$A$1:$L$16</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -1100,27 +1103,36 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1131,23 +1143,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
@@ -1700,28 +1712,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="16" t="s">
+      <c r="A1" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="C1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="D1" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="E1" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="16" t="s">
+      <c r="F1" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="G1" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="16" t="s">
+      <c r="H1" s="19" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1741,7 +1753,7 @@
       <c r="F2" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="G2" s="20" t="s">
         <v>12</v>
       </c>
       <c r="H2" t="s">
@@ -1755,13 +1767,13 @@
       <c r="B3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D3" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="17"/>
+      <c r="E3" s="20"/>
       <c r="F3" t="s">
         <v>15</v>
       </c>
@@ -1779,7 +1791,7 @@
       <c r="C4" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="17"/>
+      <c r="E4" s="20"/>
     </row>
     <row r="5" spans="1:5">
       <c r="A5">
@@ -1791,7 +1803,7 @@
       <c r="C5" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="17"/>
+      <c r="E5" s="20"/>
     </row>
     <row r="6" spans="1:8">
       <c r="A6">
@@ -1806,7 +1818,7 @@
       <c r="D6" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="20" t="s">
         <v>20</v>
       </c>
       <c r="F6" t="s">
@@ -1832,7 +1844,7 @@
       <c r="D7" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="20" t="s">
         <v>23</v>
       </c>
       <c r="F7" t="s">
@@ -1846,13 +1858,13 @@
       </c>
     </row>
     <row r="8" spans="5:5">
-      <c r="E8" s="17"/>
+      <c r="E8" s="20"/>
     </row>
     <row r="9" spans="5:5">
-      <c r="E9" s="17"/>
+      <c r="E9" s="20"/>
     </row>
     <row r="10" spans="5:5">
-      <c r="E10" s="17"/>
+      <c r="E10" s="20"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1862,557 +1874,601 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:L16"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr defaultColWidth="9.13888888888889" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="5.42592592592593" style="1" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="7" customWidth="1"/>
-    <col min="4" max="4" width="6.71296296296296" customWidth="1"/>
-    <col min="5" max="5" width="8" customWidth="1"/>
-    <col min="6" max="6" width="7.57407407407407" customWidth="1"/>
-    <col min="7" max="7" width="12.4259259259259" style="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5740740740741" style="1" customWidth="1"/>
-    <col min="9" max="9" width="7.13888888888889" style="1" customWidth="1"/>
-    <col min="10" max="10" width="11" customWidth="1"/>
-    <col min="11" max="11" width="22" customWidth="1"/>
-    <col min="12" max="12" width="20.5740740740741" customWidth="1"/>
+    <col min="1" max="1" width="5.33333333333333" style="1" customWidth="1"/>
+    <col min="2" max="2" width="21.8888888888889" style="2" customWidth="1"/>
+    <col min="3" max="3" width="11.6666666666667" style="2" customWidth="1"/>
+    <col min="4" max="4" width="10.4444444444444" style="2" customWidth="1"/>
+    <col min="5" max="5" width="15" style="2" customWidth="1"/>
+    <col min="6" max="6" width="10.1111111111111" style="2" customWidth="1"/>
+    <col min="7" max="7" width="13" style="1" customWidth="1"/>
+    <col min="8" max="8" width="11" style="1" customWidth="1"/>
+    <col min="9" max="9" width="7" style="1" customWidth="1"/>
+    <col min="10" max="10" width="10.5555555555556" style="2" customWidth="1"/>
+    <col min="11" max="11" width="28.8888888888889" style="2" customWidth="1"/>
+    <col min="12" max="12" width="19.1111111111111" style="2" customWidth="1"/>
+    <col min="13" max="16384" width="9.13888888888889" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="J1" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="K1" s="12" t="s">
+      <c r="K1" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="L1" s="12" t="s">
+      <c r="L1" s="15" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
-      <c r="A2" s="3">
+    <row r="2" hidden="1" spans="1:12">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="6">
         <v>1</v>
       </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="5">
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="7">
         <f>SUM(C2:F2)</f>
         <v>1</v>
       </c>
-      <c r="H2" s="3">
+      <c r="H2" s="4">
         <v>1</v>
       </c>
-      <c r="I2" s="3">
+      <c r="I2" s="4">
         <v>1</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4" t="str">
+      <c r="K2" s="5"/>
+      <c r="L2" s="5" t="str">
         <f>IF(AND(G2&gt;0,G2=H2),"Page completed","Yet to be completed")</f>
         <v>Page completed</v>
       </c>
     </row>
     <row r="3" spans="1:12">
-      <c r="A3" s="3">
+      <c r="A3" s="4">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="6">
         <v>1</v>
       </c>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="5">
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="7">
         <f t="shared" ref="G3:G15" si="0">SUM(C3:F3)</f>
         <v>1</v>
       </c>
-      <c r="H3" s="3">
-        <v>0</v>
-      </c>
-      <c r="I3" s="3">
-        <v>0</v>
-      </c>
-      <c r="J3" s="4" t="s">
+      <c r="H3" s="4">
+        <v>0</v>
+      </c>
+      <c r="I3" s="4">
+        <v>0</v>
+      </c>
+      <c r="J3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="K3" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="L3" s="4" t="str">
+      <c r="L3" s="5" t="str">
         <f t="shared" ref="L3:L16" si="1">IF(AND(G3&gt;0,G3=H3),"Page completed","Yet to be completed")</f>
         <v>Yet to be completed</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
-      <c r="A4" s="3">
+    <row r="4" hidden="1" spans="1:12">
+      <c r="A4" s="4">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="6">
         <v>2</v>
       </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4">
+      <c r="D4" s="6"/>
+      <c r="E4" s="6">
         <v>2</v>
       </c>
-      <c r="F4" s="4"/>
-      <c r="G4" s="5">
+      <c r="F4" s="6"/>
+      <c r="G4" s="7">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="4">
         <v>4</v>
       </c>
-      <c r="I4" s="3">
+      <c r="I4" s="4">
         <v>4</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="J4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4" t="str">
+      <c r="K4" s="5"/>
+      <c r="L4" s="5" t="str">
         <f t="shared" si="1"/>
         <v>Page completed</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
-      <c r="A5" s="3">
+    <row r="5" hidden="1" spans="1:12">
+      <c r="A5" s="4">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="5">
+      <c r="C5" s="6">
+        <v>0</v>
+      </c>
+      <c r="D5" s="6">
+        <v>0</v>
+      </c>
+      <c r="E5" s="6">
+        <v>0</v>
+      </c>
+      <c r="F5" s="6">
+        <v>0</v>
+      </c>
+      <c r="G5" s="7">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4" t="str">
+      <c r="H5" s="4">
+        <v>0</v>
+      </c>
+      <c r="I5" s="4">
+        <v>0</v>
+      </c>
+      <c r="J5" s="6"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5" t="str">
+        <f t="shared" ref="L5:L10" si="2">IF(AND(G5&gt;-1,G5=H5),"Page completed","Yet to be completed")</f>
+        <v>Page completed</v>
+      </c>
+    </row>
+    <row r="6" hidden="1" spans="1:12">
+      <c r="A6" s="4">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" s="6">
+        <v>0</v>
+      </c>
+      <c r="D6" s="6">
+        <v>0</v>
+      </c>
+      <c r="E6" s="6">
+        <v>0</v>
+      </c>
+      <c r="F6" s="6">
+        <v>0</v>
+      </c>
+      <c r="G6" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H6" s="4">
+        <v>0</v>
+      </c>
+      <c r="I6" s="4">
+        <v>0</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="L6" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>Page completed</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" s="4">
+        <v>6</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="6">
+        <v>1</v>
+      </c>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="7">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H7" s="4">
+        <v>0</v>
+      </c>
+      <c r="I7" s="4">
+        <v>0</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="L7" s="5" t="str">
+        <f>IF(AND(G7&gt;0,G7=H7),"Page completed","Yet to be completed")</f>
+        <v>Yet to be completed</v>
+      </c>
+    </row>
+    <row r="8" hidden="1" spans="1:12">
+      <c r="A8" s="4">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="6">
+        <v>1</v>
+      </c>
+      <c r="D8" s="6">
+        <v>2</v>
+      </c>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="7">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H8" s="4">
+        <v>3</v>
+      </c>
+      <c r="I8" s="4">
+        <v>3</v>
+      </c>
+      <c r="J8" s="6"/>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>Page completed</v>
+      </c>
+    </row>
+    <row r="9" hidden="1" spans="1:12">
+      <c r="A9" s="4">
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="6">
+        <v>0</v>
+      </c>
+      <c r="D9" s="6">
+        <v>0</v>
+      </c>
+      <c r="E9" s="6">
+        <v>0</v>
+      </c>
+      <c r="F9" s="6">
+        <v>0</v>
+      </c>
+      <c r="G9" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H9" s="4">
+        <v>0</v>
+      </c>
+      <c r="I9" s="4">
+        <v>0</v>
+      </c>
+      <c r="J9" s="6"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>Page completed</v>
+      </c>
+    </row>
+    <row r="10" hidden="1" spans="1:12">
+      <c r="A10" s="4">
+        <v>9</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="6">
+        <v>0</v>
+      </c>
+      <c r="D10" s="6">
+        <v>0</v>
+      </c>
+      <c r="E10" s="6">
+        <v>0</v>
+      </c>
+      <c r="F10" s="6">
+        <v>0</v>
+      </c>
+      <c r="G10" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H10" s="4">
+        <v>0</v>
+      </c>
+      <c r="I10" s="4">
+        <v>0</v>
+      </c>
+      <c r="J10" s="6"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5" t="str">
+        <f t="shared" si="2"/>
+        <v>Page completed</v>
+      </c>
+    </row>
+    <row r="11" ht="28.8" spans="1:12">
+      <c r="A11" s="4">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H11" s="4">
+        <v>0</v>
+      </c>
+      <c r="I11" s="4">
+        <v>0</v>
+      </c>
+      <c r="J11" s="6"/>
+      <c r="K11" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="L11" s="5" t="str">
         <f t="shared" si="1"/>
         <v>Yet to be completed</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
-      <c r="A6" s="3">
-        <v>5</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C6" s="4">
-        <v>0</v>
-      </c>
-      <c r="D6" s="4">
-        <v>0</v>
-      </c>
-      <c r="E6" s="4">
-        <v>0</v>
-      </c>
-      <c r="F6" s="4">
-        <v>0</v>
-      </c>
-      <c r="G6" s="5">
+    <row r="12" hidden="1" spans="1:12">
+      <c r="A12" s="4">
+        <v>11</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="6">
+        <v>0</v>
+      </c>
+      <c r="D12" s="6">
+        <v>0</v>
+      </c>
+      <c r="E12" s="6">
+        <v>0</v>
+      </c>
+      <c r="F12" s="6">
+        <v>0</v>
+      </c>
+      <c r="G12" s="7">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="3">
-        <v>0</v>
-      </c>
-      <c r="I6" s="3">
-        <v>0</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="L6" s="4" t="str">
-        <f>IF(AND(G6&gt;-1,G6=H6),"Page completed","Yet to be completed")</f>
+      <c r="H12" s="4">
+        <v>0</v>
+      </c>
+      <c r="I12" s="4">
+        <v>0</v>
+      </c>
+      <c r="J12" s="6"/>
+      <c r="K12" s="5"/>
+      <c r="L12" s="5" t="str">
+        <f>IF(AND(G12&gt;-1,G12=H12),"Page completed","Yet to be completed")</f>
         <v>Page completed</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
-      <c r="A7" s="3">
+    <row r="13" spans="1:12">
+      <c r="A13" s="4">
+        <v>12</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" s="6">
+        <v>4</v>
+      </c>
+      <c r="D13" s="6">
+        <v>3</v>
+      </c>
+      <c r="E13" s="6">
+        <v>1</v>
+      </c>
+      <c r="F13" s="6"/>
+      <c r="G13" s="7">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="H13" s="4">
+        <v>2</v>
+      </c>
+      <c r="I13" s="4">
+        <v>2</v>
+      </c>
+      <c r="J13" s="6"/>
+      <c r="K13" s="5"/>
+      <c r="L13" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>Yet to be completed</v>
+      </c>
+    </row>
+    <row r="14" ht="29.55" spans="1:12">
+      <c r="A14" s="4">
+        <v>13</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H14" s="4">
+        <v>0</v>
+      </c>
+      <c r="I14" s="4">
+        <v>0</v>
+      </c>
+      <c r="J14" s="6"/>
+      <c r="K14" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L14" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>Yet to be completed</v>
+      </c>
+    </row>
+    <row r="15" ht="15.15" hidden="1" spans="1:12">
+      <c r="A15" s="4">
+        <v>14</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" s="9">
+        <v>3</v>
+      </c>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9">
+        <v>2</v>
+      </c>
+      <c r="F15" s="9">
+        <v>1</v>
+      </c>
+      <c r="G15" s="10">
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C7" s="4">
-        <v>1</v>
-      </c>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="5">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="H7" s="3">
-        <v>0</v>
-      </c>
-      <c r="I7" s="3">
-        <v>0</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="K7" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="L7" s="4" t="str">
-        <f>IF(AND(G7&gt;0,G7=H7),"Page completed","Yet to be completed")</f>
-        <v>Yet to be completed</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12">
-      <c r="A8" s="3">
-        <v>7</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8" s="4">
-        <v>1</v>
-      </c>
-      <c r="D8" s="4">
-        <v>2</v>
-      </c>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="5">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="H8" s="3">
-        <v>3</v>
-      </c>
-      <c r="I8" s="3">
-        <v>3</v>
-      </c>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4" t="str">
+      <c r="H15" s="11">
+        <v>6</v>
+      </c>
+      <c r="I15" s="11">
+        <v>6</v>
+      </c>
+      <c r="J15" s="6"/>
+      <c r="K15" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L15" s="5" t="str">
         <f t="shared" si="1"/>
         <v>Page completed</v>
       </c>
     </row>
-    <row r="9" spans="1:12">
-      <c r="A9" s="3">
+    <row r="16" ht="15.15" spans="1:12">
+      <c r="A16" s="12"/>
+      <c r="B16" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" s="14">
+        <f>SUM(C2:C15)</f>
+        <v>13</v>
+      </c>
+      <c r="D16" s="14">
+        <f t="shared" ref="D16:I16" si="3">SUM(D2:D15)</f>
+        <v>5</v>
+      </c>
+      <c r="E16" s="14">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="F16" s="14">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="G16" s="14">
+        <f t="shared" si="3"/>
+        <v>24</v>
+      </c>
+      <c r="H16" s="14">
+        <f t="shared" si="3"/>
+        <v>16</v>
+      </c>
+      <c r="I16" s="17">
+        <f t="shared" si="3"/>
+        <v>16</v>
+      </c>
+      <c r="J16" s="18"/>
+      <c r="K16" s="6"/>
+      <c r="L16" s="6"/>
+    </row>
+    <row r="17" spans="7:7">
+      <c r="G17" s="1">
+        <f>G16-H16</f>
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" s="4">
-        <v>0</v>
-      </c>
-      <c r="D9" s="4">
-        <v>0</v>
-      </c>
-      <c r="E9" s="4">
-        <v>0</v>
-      </c>
-      <c r="F9" s="4">
-        <v>0</v>
-      </c>
-      <c r="G9" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H9" s="3">
-        <v>0</v>
-      </c>
-      <c r="I9" s="3">
-        <v>0</v>
-      </c>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
-      <c r="L9" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Yet to be completed</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12">
-      <c r="A10" s="3">
-        <v>9</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" s="4">
-        <v>0</v>
-      </c>
-      <c r="D10" s="4">
-        <v>0</v>
-      </c>
-      <c r="E10" s="4">
-        <v>0</v>
-      </c>
-      <c r="F10" s="4">
-        <v>0</v>
-      </c>
-      <c r="G10" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H10" s="3">
-        <v>0</v>
-      </c>
-      <c r="I10" s="3">
-        <v>0</v>
-      </c>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
-      <c r="L10" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Yet to be completed</v>
-      </c>
-    </row>
-    <row r="11" ht="28.8" spans="1:12">
-      <c r="A11" s="3">
-        <v>10</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H11" s="3">
-        <v>0</v>
-      </c>
-      <c r="I11" s="3">
-        <v>0</v>
-      </c>
-      <c r="J11" s="4"/>
-      <c r="K11" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="L11" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Yet to be completed</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12">
-      <c r="A12" s="3">
-        <v>11</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H12" s="3">
-        <v>0</v>
-      </c>
-      <c r="I12" s="3">
-        <v>0</v>
-      </c>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
-      <c r="L12" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Yet to be completed</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12">
-      <c r="A13" s="3">
-        <v>12</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H13" s="3">
-        <v>0</v>
-      </c>
-      <c r="I13" s="3">
-        <v>0</v>
-      </c>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4"/>
-      <c r="L13" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Yet to be completed</v>
-      </c>
-    </row>
-    <row r="14" ht="28.8" spans="1:12">
-      <c r="A14" s="3">
-        <v>13</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H14" s="3">
-        <v>0</v>
-      </c>
-      <c r="I14" s="3">
-        <v>0</v>
-      </c>
-      <c r="J14" s="4"/>
-      <c r="K14" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="L14" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Yet to be completed</v>
-      </c>
-    </row>
-    <row r="15" ht="15.15" spans="1:12">
-      <c r="A15" s="3">
-        <v>14</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="C15" s="6">
-        <v>3</v>
-      </c>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6">
-        <v>2</v>
-      </c>
-      <c r="F15" s="6">
-        <v>1</v>
-      </c>
-      <c r="G15" s="7">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="H15" s="8">
-        <v>6</v>
-      </c>
-      <c r="I15" s="8">
-        <v>6</v>
-      </c>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="L15" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>Page completed</v>
-      </c>
-    </row>
-    <row r="16" ht="15.15" spans="1:12">
-      <c r="A16" s="9"/>
-      <c r="B16" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="C16" s="11">
-        <f>SUM(C2:C15)</f>
-        <v>9</v>
-      </c>
-      <c r="D16" s="11">
-        <f t="shared" ref="D16:I16" si="2">SUM(D2:D15)</f>
-        <v>2</v>
-      </c>
-      <c r="E16" s="11">
-        <f t="shared" si="2"/>
-        <v>4</v>
-      </c>
-      <c r="F16" s="11">
-        <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-      <c r="G16" s="11">
-        <f t="shared" si="2"/>
-        <v>16</v>
-      </c>
-      <c r="H16" s="11">
-        <f t="shared" si="2"/>
-        <v>14</v>
-      </c>
-      <c r="I16" s="14">
-        <f t="shared" si="2"/>
-        <v>14</v>
-      </c>
-      <c r="J16" s="15"/>
-      <c r="K16" s="4"/>
-      <c r="L16" s="4"/>
     </row>
   </sheetData>
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:L16" etc:filterBottomFollowUsedRange="0">
+    <filterColumn colId="11">
+      <filters blank="1">
+        <filter val="Yet to be completed"/>
+      </filters>
+    </filterColumn>
+    <extLst/>
+  </autoFilter>
   <sortState ref="B3:B15">
     <sortCondition ref="B3"/>
   </sortState>
+  <mergeCells count="1">
+    <mergeCell ref="G17:H17"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>

</xml_diff>

<commit_message>
Student Details Page Completed?
</commit_message>
<xml_diff>
--- a/Zenskar_MAMS/Helpers/Queries.xlsx
+++ b/Zenskar_MAMS/Helpers/Queries.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8280" activeTab="1"/>
+    <workbookView windowWidth="23040" windowHeight="9000" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2320,18 +2320,18 @@
         <v>9</v>
       </c>
       <c r="H13" s="3">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I13" s="3">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="K13" s="4"/>
       <c r="L13" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Yet to be completed</v>
+        <v>Page completed</v>
       </c>
     </row>
     <row r="14" ht="29.55" spans="1:12">
@@ -2427,11 +2427,11 @@
       </c>
       <c r="H16" s="11">
         <f t="shared" si="3"/>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I16" s="13">
         <f t="shared" si="3"/>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J16" s="14"/>
       <c r="K16" s="3"/>
@@ -2440,7 +2440,7 @@
     <row r="17" spans="7:7">
       <c r="G17" s="1">
         <f>G16-H16</f>
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
StudentsList Case Query Update
</commit_message>
<xml_diff>
--- a/Zenskar_MAMS/Helpers/Queries.xlsx
+++ b/Zenskar_MAMS/Helpers/Queries.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="111">
   <si>
     <t>Slno</t>
   </si>
@@ -190,8 +190,8 @@
     <t>StudentsList</t>
   </si>
   <si>
-    <t xml:space="preserve">Has Case in the Query
-</t>
+    <t>Has Case in the Query
+Got the Data from DB and then used the case</t>
   </si>
   <si>
     <t>UserManagement</t>
@@ -2299,7 +2299,7 @@
         <v>Page completed</v>
       </c>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" hidden="1" spans="1:12">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -2334,28 +2334,38 @@
         <v>Page completed</v>
       </c>
     </row>
-    <row r="14" ht="29.55" spans="1:12">
+    <row r="14" ht="43.95" spans="1:12">
       <c r="A14" s="3">
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
+      <c r="C14" s="3">
+        <v>1</v>
+      </c>
+      <c r="D14" s="3">
+        <v>1</v>
+      </c>
+      <c r="E14" s="3">
+        <v>2</v>
+      </c>
+      <c r="F14" s="3">
+        <v>1</v>
+      </c>
       <c r="G14" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>SUM(C14:F14)</f>
+        <v>5</v>
       </c>
       <c r="H14" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14" s="3">
-        <v>0</v>
-      </c>
-      <c r="J14" s="3"/>
+        <v>1</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="K14" s="12" t="s">
         <v>49</v>
       </c>
@@ -2364,7 +2374,7 @@
         <v>Yet to be completed</v>
       </c>
     </row>
-    <row r="15" ht="15.15" hidden="1" spans="1:12">
+    <row r="15" hidden="1" spans="1:12">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -2400,38 +2410,38 @@
         <v>Page completed</v>
       </c>
     </row>
-    <row r="16" ht="15.15" spans="1:12">
+    <row r="16" spans="1:12">
       <c r="A16" s="9"/>
       <c r="B16" s="10" t="s">
         <v>52</v>
       </c>
       <c r="C16" s="11">
         <f>SUM(C2:C15)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D16" s="11">
         <f t="shared" ref="D16:I16" si="3">SUM(D2:D15)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E16" s="11">
         <f t="shared" si="3"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F16" s="11">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G16" s="11">
         <f t="shared" si="3"/>
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="H16" s="11">
         <f t="shared" si="3"/>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I16" s="13">
         <f t="shared" si="3"/>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J16" s="14"/>
       <c r="K16" s="3"/>
@@ -2440,7 +2450,7 @@
     <row r="17" spans="7:7">
       <c r="G17" s="1">
         <f>G16-H16</f>
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Completed StudentsList, and all Home pages rewrite
</commit_message>
<xml_diff>
--- a/Zenskar_MAMS/Helpers/Queries.xlsx
+++ b/Zenskar_MAMS/Helpers/Queries.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000" activeTab="1"/>
+    <workbookView windowWidth="23040" windowHeight="8280" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1874,7 +1874,7 @@
     <col min="6" max="6" width="10.1111111111111" style="1" customWidth="1"/>
     <col min="7" max="7" width="13" style="1" customWidth="1"/>
     <col min="8" max="8" width="11" style="1" customWidth="1"/>
-    <col min="9" max="9" width="7" style="1" customWidth="1"/>
+    <col min="9" max="9" width="8.44444444444444" style="1" customWidth="1"/>
     <col min="10" max="10" width="10.5555555555556" style="1" customWidth="1"/>
     <col min="11" max="11" width="28.8888888888889" style="1" customWidth="1"/>
     <col min="12" max="12" width="19.1111111111111" style="1" customWidth="1"/>
@@ -1969,10 +1969,10 @@
         <v>1</v>
       </c>
       <c r="H3" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" s="3" t="s">
         <v>15</v>
@@ -1982,7 +1982,7 @@
       </c>
       <c r="L3" s="4" t="str">
         <f t="shared" ref="L3:L16" si="1">IF(AND(G3&gt;0,G3=H3),"Page completed","Yet to be completed")</f>
-        <v>Yet to be completed</v>
+        <v>Page completed</v>
       </c>
     </row>
     <row r="4" hidden="1" spans="1:12">
@@ -2095,7 +2095,7 @@
         <v>Page completed</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" hidden="1" spans="1:12">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -2113,10 +2113,10 @@
         <v>1</v>
       </c>
       <c r="H7" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7" s="3" t="s">
         <v>15</v>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="L7" s="4" t="str">
         <f>IF(AND(G7&gt;0,G7=H7),"Page completed","Yet to be completed")</f>
-        <v>Yet to be completed</v>
+        <v>Page completed</v>
       </c>
     </row>
     <row r="8" hidden="1" spans="1:12">
@@ -2233,7 +2233,7 @@
         <v>Page completed</v>
       </c>
     </row>
-    <row r="11" ht="28.8" spans="1:12">
+    <row r="11" ht="29.55" spans="1:12">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -2334,7 +2334,7 @@
         <v>Page completed</v>
       </c>
     </row>
-    <row r="14" ht="43.95" spans="1:12">
+    <row r="14" ht="43.2" hidden="1" spans="1:12">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -2358,10 +2358,10 @@
         <v>5</v>
       </c>
       <c r="H14" s="3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I14" s="3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J14" s="3" t="s">
         <v>11</v>
@@ -2371,10 +2371,10 @@
       </c>
       <c r="L14" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Yet to be completed</v>
-      </c>
-    </row>
-    <row r="15" hidden="1" spans="1:12">
+        <v>Page completed</v>
+      </c>
+    </row>
+    <row r="15" ht="15.15" hidden="1" spans="1:12">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -2437,11 +2437,11 @@
       </c>
       <c r="H16" s="11">
         <f t="shared" si="3"/>
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="I16" s="13">
         <f t="shared" si="3"/>
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="J16" s="14"/>
       <c r="K16" s="3"/>
@@ -2450,16 +2450,15 @@
     <row r="17" spans="7:7">
       <c r="G17" s="1">
         <f>G16-H16</f>
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:L17" etc:filterBottomFollowUsedRange="0">
     <filterColumn colId="11">
-      <customFilters>
-        <customFilter operator="equal" val=""/>
-        <customFilter operator="equal" val="Yet to be completed"/>
-      </customFilters>
+      <filters blank="1">
+        <filter val="Yet to be completed"/>
+      </filters>
     </filterColumn>
     <extLst/>
   </autoFilter>

</xml_diff>

<commit_message>
Added Location and Belt List to DB
</commit_message>
<xml_diff>
--- a/Zenskar_MAMS/Helpers/Queries.xlsx
+++ b/Zenskar_MAMS/Helpers/Queries.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8280" activeTab="1"/>
+    <workbookView windowWidth="28800" windowHeight="11460" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="110">
   <si>
     <t>Slno</t>
   </si>
@@ -154,9 +154,6 @@
   </si>
   <si>
     <t>InstructorHome</t>
-  </si>
-  <si>
-    <t>NA</t>
   </si>
   <si>
     <t>No Queries</t>
@@ -1689,14 +1686,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:H10"/>
-  <sheetFormatPr defaultColWidth="9.13888888888889" defaultRowHeight="14.4" outlineLevelCol="7"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="7"/>
   <cols>
-    <col min="2" max="2" width="13.5740740740741" customWidth="1"/>
-    <col min="3" max="3" width="110.574074074074" customWidth="1"/>
-    <col min="4" max="4" width="11.4259259259259" customWidth="1"/>
-    <col min="5" max="5" width="28.8611111111111" customWidth="1"/>
+    <col min="2" max="2" width="13.5714285714286" customWidth="1"/>
+    <col min="3" max="3" width="110.571428571429" customWidth="1"/>
+    <col min="4" max="4" width="11.4285714285714" customWidth="1"/>
+    <col min="5" max="5" width="28.8571428571429" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
-    <col min="7" max="7" width="17.5740740740741" customWidth="1"/>
+    <col min="7" max="7" width="17.5714285714286" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -1725,7 +1722,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" ht="28.8" spans="1:8">
+    <row r="2" ht="30" spans="1:8">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1748,7 +1745,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" ht="129.6" spans="1:8">
+    <row r="3" ht="135" spans="1:8">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1819,7 +1816,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" ht="28.8" spans="1:8">
+    <row r="7" ht="30" spans="1:8">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1862,23 +1859,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr filterMode="1"/>
+  <sheetPr/>
   <dimension ref="A1:L17"/>
-  <sheetFormatPr defaultColWidth="9.13888888888889" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.33333333333333" style="1" customWidth="1"/>
-    <col min="2" max="2" width="21.8888888888889" style="1" customWidth="1"/>
+    <col min="2" max="2" width="21.8857142857143" style="1" customWidth="1"/>
     <col min="3" max="3" width="11.6666666666667" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10.4444444444444" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.447619047619" style="1" customWidth="1"/>
     <col min="5" max="5" width="15" style="1" customWidth="1"/>
-    <col min="6" max="6" width="10.1111111111111" style="1" customWidth="1"/>
+    <col min="6" max="6" width="10.1142857142857" style="1" customWidth="1"/>
     <col min="7" max="7" width="13" style="1" customWidth="1"/>
     <col min="8" max="8" width="11" style="1" customWidth="1"/>
-    <col min="9" max="9" width="8.44444444444444" style="1" customWidth="1"/>
-    <col min="10" max="10" width="10.5555555555556" style="1" customWidth="1"/>
-    <col min="11" max="11" width="28.8888888888889" style="1" customWidth="1"/>
-    <col min="12" max="12" width="19.1111111111111" style="1" customWidth="1"/>
-    <col min="13" max="16384" width="9.13888888888889" style="1"/>
+    <col min="9" max="9" width="8.44761904761905" style="1" customWidth="1"/>
+    <col min="10" max="10" width="10.552380952381" style="1" customWidth="1"/>
+    <col min="11" max="11" width="28.8857142857143" style="1" customWidth="1"/>
+    <col min="12" max="12" width="19.1142857142857" style="1" customWidth="1"/>
+    <col min="13" max="16384" width="9.14285714285714" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -1919,7 +1916,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" hidden="1" spans="1:12">
+    <row r="2" spans="1:12">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -1951,7 +1948,7 @@
         <v>Page completed</v>
       </c>
     </row>
-    <row r="3" hidden="1" spans="1:12">
+    <row r="3" spans="1:12">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -1985,7 +1982,7 @@
         <v>Page completed</v>
       </c>
     </row>
-    <row r="4" hidden="1" spans="1:12">
+    <row r="4" spans="1:12">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -2011,7 +2008,7 @@
         <v>4</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="K4" s="4"/>
       <c r="L4" s="4" t="str">
@@ -2019,7 +2016,7 @@
         <v>Page completed</v>
       </c>
     </row>
-    <row r="5" hidden="1" spans="1:12">
+    <row r="5" spans="1:12">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -2048,14 +2045,16 @@
       <c r="I5" s="3">
         <v>0</v>
       </c>
-      <c r="J5" s="3"/>
+      <c r="J5" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="K5" s="4"/>
       <c r="L5" s="4" t="str">
         <f t="shared" ref="L5:L10" si="2">IF(AND(G5&gt;-1,G5=H5),"Page completed","Yet to be completed")</f>
         <v>Page completed</v>
       </c>
     </row>
-    <row r="6" hidden="1" spans="1:12">
+    <row r="6" spans="1:12">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -2085,22 +2084,22 @@
         <v>0</v>
       </c>
       <c r="J6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="K6" s="4" t="s">
         <v>38</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="L6" s="4" t="str">
         <f t="shared" si="2"/>
         <v>Page completed</v>
       </c>
     </row>
-    <row r="7" hidden="1" spans="1:12">
+    <row r="7" spans="1:12">
       <c r="A7" s="3">
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C7" s="3">
         <v>1</v>
@@ -2119,7 +2118,7 @@
         <v>1</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="K7" s="4" t="s">
         <v>35</v>
@@ -2129,12 +2128,12 @@
         <v>Page completed</v>
       </c>
     </row>
-    <row r="8" hidden="1" spans="1:12">
+    <row r="8" spans="1:12">
       <c r="A8" s="3">
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C8" s="3">
         <v>1</v>
@@ -2154,19 +2153,21 @@
       <c r="I8" s="3">
         <v>3</v>
       </c>
-      <c r="J8" s="3"/>
+      <c r="J8" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="K8" s="4"/>
       <c r="L8" s="4" t="str">
         <f t="shared" si="1"/>
         <v>Page completed</v>
       </c>
     </row>
-    <row r="9" hidden="1" spans="1:12">
+    <row r="9" spans="1:12">
       <c r="A9" s="3">
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C9" s="3">
         <v>0</v>
@@ -2190,19 +2191,21 @@
       <c r="I9" s="3">
         <v>0</v>
       </c>
-      <c r="J9" s="3"/>
+      <c r="J9" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="K9" s="4"/>
       <c r="L9" s="4" t="str">
         <f t="shared" si="2"/>
         <v>Page completed</v>
       </c>
     </row>
-    <row r="10" hidden="1" spans="1:12">
+    <row r="10" spans="1:12">
       <c r="A10" s="3">
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C10" s="3">
         <v>0</v>
@@ -2226,19 +2229,21 @@
       <c r="I10" s="3">
         <v>0</v>
       </c>
-      <c r="J10" s="3"/>
+      <c r="J10" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="K10" s="4"/>
       <c r="L10" s="4" t="str">
         <f t="shared" si="2"/>
         <v>Page completed</v>
       </c>
     </row>
-    <row r="11" ht="29.55" spans="1:12">
+    <row r="11" ht="30" spans="1:12">
       <c r="A11" s="3">
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
@@ -2248,26 +2253,28 @@
         <v>9</v>
       </c>
       <c r="H11" s="3">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I11" s="3">
-        <v>0</v>
-      </c>
-      <c r="J11" s="3"/>
+        <v>9</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="K11" s="12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="L11" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Yet to be completed</v>
-      </c>
-    </row>
-    <row r="12" hidden="1" spans="1:12">
+        <v>Page completed</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
       <c r="A12" s="3">
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C12" s="3">
         <v>0</v>
@@ -2291,19 +2298,21 @@
       <c r="I12" s="3">
         <v>0</v>
       </c>
-      <c r="J12" s="3"/>
+      <c r="J12" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="K12" s="4"/>
       <c r="L12" s="4" t="str">
         <f>IF(AND(G12&gt;-1,G12=H12),"Page completed","Yet to be completed")</f>
         <v>Page completed</v>
       </c>
     </row>
-    <row r="13" hidden="1" spans="1:12">
+    <row r="13" spans="1:12">
       <c r="A13" s="3">
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C13" s="3">
         <v>4</v>
@@ -2333,12 +2342,12 @@
         <v>Page completed</v>
       </c>
     </row>
-    <row r="14" ht="43.2" hidden="1" spans="1:12">
+    <row r="14" ht="45" spans="1:12">
       <c r="A14" s="3">
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C14" s="3">
         <v>1</v>
@@ -2366,19 +2375,19 @@
         <v>11</v>
       </c>
       <c r="K14" s="12" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L14" s="4" t="str">
         <f t="shared" si="1"/>
         <v>Page completed</v>
       </c>
     </row>
-    <row r="15" ht="15.15" hidden="1" spans="1:12">
+    <row r="15" ht="15.75" spans="1:12">
       <c r="A15" s="3">
         <v>14</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C15" s="7">
         <v>3</v>
@@ -2400,19 +2409,21 @@
       <c r="I15" s="7">
         <v>6</v>
       </c>
-      <c r="J15" s="3"/>
+      <c r="J15" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="K15" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="L15" s="4" t="str">
         <f t="shared" si="1"/>
         <v>Page completed</v>
       </c>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" ht="15.75" spans="1:12">
       <c r="A16" s="9"/>
       <c r="B16" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C16" s="11">
         <f>SUM(C2:C15)</f>
@@ -2436,11 +2447,11 @@
       </c>
       <c r="H16" s="11">
         <f t="shared" si="3"/>
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="I16" s="13">
         <f t="shared" si="3"/>
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="J16" s="14"/>
       <c r="K16" s="3"/>
@@ -2449,18 +2460,10 @@
     <row r="17" spans="7:7">
       <c r="G17" s="1">
         <f>G16-H16</f>
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:L17" etc:filterBottomFollowUsedRange="0">
-    <filterColumn colId="11">
-      <filters blank="1">
-        <filter val="Yet to be completed"/>
-      </filters>
-    </filterColumn>
-    <extLst/>
-  </autoFilter>
   <sortState ref="B3:B15">
     <sortCondition ref="B3"/>
   </sortState>
@@ -2476,14 +2479,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F42"/>
-  <sheetFormatPr defaultColWidth="10.287037037037" defaultRowHeight="14.4" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="10.2857142857143" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="5.42592592592593" customWidth="1"/>
-    <col min="2" max="2" width="52.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="5.42857142857143" customWidth="1"/>
+    <col min="2" max="2" width="52.7142857142857" customWidth="1"/>
     <col min="3" max="3" width="62.3333333333333" customWidth="1"/>
-    <col min="4" max="4" width="16.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="12.712962962963" customWidth="1"/>
-    <col min="6" max="6" width="5.13888888888889" customWidth="1"/>
+    <col min="4" max="4" width="16.7142857142857" customWidth="1"/>
+    <col min="5" max="5" width="12.7142857142857" customWidth="1"/>
+    <col min="6" max="6" width="5.14285714285714" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" spans="1:5">
@@ -2500,7 +2503,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -2508,19 +2511,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C2" t="s">
         <v>54</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>55</v>
       </c>
-      <c r="D2" t="s">
-        <v>56</v>
-      </c>
       <c r="E2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -2528,19 +2531,19 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" t="s">
         <v>59</v>
       </c>
-      <c r="D3" t="s">
-        <v>60</v>
-      </c>
       <c r="E3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -2548,19 +2551,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" t="s">
         <v>61</v>
       </c>
-      <c r="D4" t="s">
-        <v>62</v>
-      </c>
       <c r="E4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -2568,19 +2571,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -2588,19 +2591,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -2608,19 +2611,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D7" t="s">
         <v>65</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>66</v>
       </c>
-      <c r="E7" t="s">
-        <v>67</v>
-      </c>
       <c r="F7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -2628,19 +2631,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C8" t="s">
         <v>68</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>69</v>
       </c>
-      <c r="D8" t="s">
-        <v>70</v>
-      </c>
       <c r="E8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -2648,19 +2651,19 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C9" t="s">
         <v>19</v>
       </c>
       <c r="D9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -2668,19 +2671,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2688,19 +2691,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C11" t="s">
         <v>73</v>
       </c>
-      <c r="C11" t="s">
-        <v>74</v>
-      </c>
       <c r="D11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2708,19 +2711,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C12" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -2728,19 +2731,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C13" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E13" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -2748,19 +2751,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14" t="s">
         <v>77</v>
       </c>
-      <c r="C14" t="s">
-        <v>78</v>
-      </c>
       <c r="D14" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E14" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F14" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -2768,19 +2771,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F15" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -2788,19 +2791,19 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C16" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -2808,19 +2811,19 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D17" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E17" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F17" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -2828,19 +2831,19 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C18" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D18" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E18" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F18" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -2848,19 +2851,19 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C19" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D19" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E19" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F19" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -2868,19 +2871,19 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C20" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D20" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E20" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F20" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -2888,19 +2891,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C21" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D21" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E21" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F21" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -2908,19 +2911,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C22" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D22" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E22" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F22" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -2928,19 +2931,19 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
+        <v>86</v>
+      </c>
+      <c r="C23" t="s">
         <v>87</v>
       </c>
-      <c r="C23" t="s">
-        <v>88</v>
-      </c>
       <c r="D23" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E23" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -2948,19 +2951,19 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C24" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F24" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -2968,19 +2971,19 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C25" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -2988,19 +2991,19 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C26" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D26" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E26" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F26" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -3008,19 +3011,19 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C27" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D27" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E27" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F27" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -3028,19 +3031,19 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C28" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D28" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E28" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F28" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -3048,19 +3051,19 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C29" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D29" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E29" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F29" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -3068,19 +3071,19 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C30" t="s">
+        <v>93</v>
+      </c>
+      <c r="D30" t="s">
         <v>94</v>
       </c>
-      <c r="D30" t="s">
-        <v>95</v>
-      </c>
       <c r="E30" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F30" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -3088,19 +3091,19 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
+        <v>95</v>
+      </c>
+      <c r="C31" t="s">
         <v>96</v>
       </c>
-      <c r="C31" t="s">
-        <v>97</v>
-      </c>
       <c r="D31" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E31" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F31" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -3108,19 +3111,19 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C32" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D32" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E32" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F32" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -3128,19 +3131,19 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C33" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D33" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E33" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F33" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -3148,19 +3151,19 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C34" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D34" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E34" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F34" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -3168,19 +3171,19 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C35" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D35" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E35" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F35" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -3188,19 +3191,19 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C36" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D36" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E36" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F36" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -3208,19 +3211,19 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
+        <v>102</v>
+      </c>
+      <c r="C37" t="s">
         <v>103</v>
       </c>
-      <c r="C37" t="s">
-        <v>104</v>
-      </c>
       <c r="D37" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E37" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F37" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -3228,19 +3231,19 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C38" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D38" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E38" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F38" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -3248,19 +3251,19 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C39" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D39" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E39" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F39" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -3268,19 +3271,19 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
+        <v>106</v>
+      </c>
+      <c r="C40" t="s">
         <v>107</v>
       </c>
-      <c r="C40" t="s">
-        <v>108</v>
-      </c>
       <c r="D40" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E40" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F40" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -3288,19 +3291,19 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C41" t="s">
+        <v>93</v>
+      </c>
+      <c r="D41" t="s">
         <v>94</v>
       </c>
-      <c r="D41" t="s">
-        <v>95</v>
-      </c>
       <c r="E41" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F41" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -3308,19 +3311,19 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
+        <v>108</v>
+      </c>
+      <c r="C42" t="s">
         <v>109</v>
       </c>
-      <c r="C42" t="s">
-        <v>110</v>
-      </c>
       <c r="D42" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E42" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F42" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>